<commit_message>
data(catalogs): synchronize master 22-sheet catalogs, running knowledge charters, and daily snapshots
- Rebuild and certify master 22-sheet Excel workbooks and companion JSONs for all 10 registered products
- Compile and deduplicate 165 total active rules in outputs/history/master_knowledge_registry.json
- Generate outputs/history/running_knowledge_charter.md (51 KB) for shared Google Doc synchronization
- Record stable daily snapshot catalog_2026-09-13.json per active product (INV-6)
- Update product-specific Markdown sync payloads across all portfolio directories
</commit_message>
<xml_diff>
--- a/outputs/Alletra/Storage/Alletra_Storage_System/Alletra_Storage_System_OCA_Catalog.xlsx
+++ b/outputs/Alletra/Storage/Alletra_Storage_System/Alletra_Storage_System_OCA_Catalog.xlsx
@@ -13,11 +13,11 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Category Summary'!A1:H2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'All SKUs'!A1:X4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'All SKUs'!A1:AC4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2">'Chassis Variants'!A1:K4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3">'Rules &amp; Constraints'!A1:E3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4">'Price History Timeline'!A1:G4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5">'Chassis'!A1:X4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5">'Chassis'!A1:AC4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6">'Metadata'!A1:B21</definedName>
   </definedNames>
 </workbook>
@@ -561,7 +561,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X4"/>
+  <dimension ref="A1:AC4"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="35.83203125" customWidth="1"/>
@@ -580,13 +580,18 @@
     <col min="15" max="15" width="18.83203125" customWidth="1"/>
     <col min="16" max="16" width="15.83203125" customWidth="1"/>
     <col min="17" max="17" width="14.83203125" customWidth="1"/>
-    <col min="18" max="18" width="12.83203125" customWidth="1"/>
-    <col min="19" max="19" width="16.83203125" customWidth="1"/>
-    <col min="20" max="20" width="16.83203125" customWidth="1"/>
-    <col min="21" max="21" width="22.83203125" customWidth="1"/>
-    <col min="22" max="22" width="18.83203125" customWidth="1"/>
+    <col min="18" max="18" width="24.83203125" customWidth="1"/>
+    <col min="19" max="19" width="18.83203125" customWidth="1"/>
+    <col min="20" max="20" width="24.83203125" customWidth="1"/>
+    <col min="21" max="21" width="20.83203125" customWidth="1"/>
+    <col min="22" max="22" width="12.83203125" customWidth="1"/>
     <col min="23" max="23" width="16.83203125" customWidth="1"/>
-    <col min="24" max="24" width="55.83203125" customWidth="1"/>
+    <col min="24" max="24" width="60.83203125" customWidth="1"/>
+    <col min="25" max="25" width="16.83203125" customWidth="1"/>
+    <col min="26" max="26" width="22.83203125" customWidth="1"/>
+    <col min="27" max="27" width="18.83203125" customWidth="1"/>
+    <col min="28" max="28" width="16.83203125" customWidth="1"/>
+    <col min="29" max="29" width="55.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -642,24 +647,39 @@
         <v>HPE Recommended</v>
       </c>
       <c r="R1" s="3" t="str">
+        <v>Availability</v>
+      </c>
+      <c r="S1" s="3" t="str">
+        <v>Lead Time</v>
+      </c>
+      <c r="T1" s="3" t="str">
+        <v>Lead Time Source</v>
+      </c>
+      <c r="U1" s="3" t="str">
+        <v>Lifecycle Status</v>
+      </c>
+      <c r="V1" s="3" t="str">
         <v>Start Date</v>
       </c>
-      <c r="S1" s="3" t="str">
+      <c r="W1" s="3" t="str">
         <v>Discontinued Date</v>
       </c>
-      <c r="T1" s="3" t="str">
+      <c r="X1" s="3" t="str">
+        <v>Vendor Attributes (JSON)</v>
+      </c>
+      <c r="Y1" s="3" t="str">
         <v>Diff Status</v>
       </c>
-      <c r="U1" s="3" t="str">
+      <c r="Z1" s="3" t="str">
         <v>Previous List Price (USD)</v>
       </c>
-      <c r="V1" s="3" t="str">
+      <c r="AA1" s="3" t="str">
         <v>Price Change (USD)</v>
       </c>
-      <c r="W1" s="3" t="str">
+      <c r="AB1" s="3" t="str">
         <v>Price Change (%)</v>
       </c>
-      <c r="X1" s="3" t="str">
+      <c r="AC1" s="3" t="str">
         <v>Price History Trail</v>
       </c>
     </row>
@@ -716,24 +736,39 @@
         <v>Yes</v>
       </c>
       <c r="R2" s="2" t="str">
+        <v/>
+      </c>
+      <c r="S2" s="2" t="str">
+        <v/>
+      </c>
+      <c r="T2" s="2" t="str">
+        <v/>
+      </c>
+      <c r="U2" s="2" t="str">
+        <v/>
+      </c>
+      <c r="V2" s="2" t="str">
         <v>—</v>
       </c>
-      <c r="S2" s="2" t="str">
-        <v/>
-      </c>
-      <c r="T2" s="2" t="str">
+      <c r="W2" s="2" t="str">
+        <v/>
+      </c>
+      <c r="X2" s="2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" s="2" t="str">
         <v>UNCHANGED</v>
       </c>
-      <c r="U2" s="6">
+      <c r="Z2" s="6">
         <v>12500</v>
       </c>
-      <c r="V2" s="6">
-        <v>0</v>
-      </c>
-      <c r="W2" s="6">
-        <v>0</v>
-      </c>
-      <c r="X2" s="6">
+      <c r="AA2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC2" s="6">
         <v>2026</v>
       </c>
     </row>
@@ -790,24 +825,39 @@
         <v>Yes</v>
       </c>
       <c r="R3" s="2" t="str">
+        <v/>
+      </c>
+      <c r="S3" s="2" t="str">
+        <v/>
+      </c>
+      <c r="T3" s="2" t="str">
+        <v/>
+      </c>
+      <c r="U3" s="2" t="str">
+        <v/>
+      </c>
+      <c r="V3" s="2" t="str">
         <v>—</v>
       </c>
-      <c r="S3" s="2" t="str">
-        <v/>
-      </c>
-      <c r="T3" s="2" t="str">
+      <c r="W3" s="2" t="str">
+        <v/>
+      </c>
+      <c r="X3" s="2" t="str">
+        <v/>
+      </c>
+      <c r="Y3" s="2" t="str">
         <v>UNCHANGED</v>
       </c>
-      <c r="U3" s="6">
+      <c r="Z3" s="6">
         <v>18900</v>
       </c>
-      <c r="V3" s="6">
-        <v>0</v>
-      </c>
-      <c r="W3" s="6">
-        <v>0</v>
-      </c>
-      <c r="X3" s="6">
+      <c r="AA3" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC3" s="6">
         <v>2026</v>
       </c>
     </row>
@@ -864,31 +914,46 @@
         <v>Yes</v>
       </c>
       <c r="R4" s="2" t="str">
+        <v/>
+      </c>
+      <c r="S4" s="2" t="str">
+        <v/>
+      </c>
+      <c r="T4" s="2" t="str">
+        <v/>
+      </c>
+      <c r="U4" s="2" t="str">
+        <v/>
+      </c>
+      <c r="V4" s="2" t="str">
         <v>—</v>
       </c>
-      <c r="S4" s="2" t="str">
-        <v/>
-      </c>
-      <c r="T4" s="2" t="str">
+      <c r="W4" s="2" t="str">
+        <v/>
+      </c>
+      <c r="X4" s="2" t="str">
+        <v/>
+      </c>
+      <c r="Y4" s="2" t="str">
         <v>UNCHANGED</v>
       </c>
-      <c r="U4" s="6">
+      <c r="Z4" s="6">
         <v>15200</v>
       </c>
-      <c r="V4" s="6">
-        <v>0</v>
-      </c>
-      <c r="W4" s="6">
-        <v>0</v>
-      </c>
-      <c r="X4" s="6">
+      <c r="AA4" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="6">
         <v>2026</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X4"/>
+  <autoFilter ref="A1:AC4"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:X4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1243,7 +1308,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X4"/>
+  <dimension ref="A1:AC4"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="35.83203125" customWidth="1"/>
@@ -1262,13 +1327,18 @@
     <col min="15" max="15" width="18.83203125" customWidth="1"/>
     <col min="16" max="16" width="15.83203125" customWidth="1"/>
     <col min="17" max="17" width="14.83203125" customWidth="1"/>
-    <col min="18" max="18" width="12.83203125" customWidth="1"/>
-    <col min="19" max="19" width="16.83203125" customWidth="1"/>
-    <col min="20" max="20" width="16.83203125" customWidth="1"/>
-    <col min="21" max="21" width="22.83203125" customWidth="1"/>
-    <col min="22" max="22" width="18.83203125" customWidth="1"/>
+    <col min="18" max="18" width="24.83203125" customWidth="1"/>
+    <col min="19" max="19" width="18.83203125" customWidth="1"/>
+    <col min="20" max="20" width="24.83203125" customWidth="1"/>
+    <col min="21" max="21" width="20.83203125" customWidth="1"/>
+    <col min="22" max="22" width="12.83203125" customWidth="1"/>
     <col min="23" max="23" width="16.83203125" customWidth="1"/>
-    <col min="24" max="24" width="55.83203125" customWidth="1"/>
+    <col min="24" max="24" width="60.83203125" customWidth="1"/>
+    <col min="25" max="25" width="16.83203125" customWidth="1"/>
+    <col min="26" max="26" width="22.83203125" customWidth="1"/>
+    <col min="27" max="27" width="18.83203125" customWidth="1"/>
+    <col min="28" max="28" width="16.83203125" customWidth="1"/>
+    <col min="29" max="29" width="55.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1324,24 +1394,39 @@
         <v>HPE Recommended</v>
       </c>
       <c r="R1" s="3" t="str">
+        <v>Availability</v>
+      </c>
+      <c r="S1" s="3" t="str">
+        <v>Lead Time</v>
+      </c>
+      <c r="T1" s="3" t="str">
+        <v>Lead Time Source</v>
+      </c>
+      <c r="U1" s="3" t="str">
+        <v>Lifecycle Status</v>
+      </c>
+      <c r="V1" s="3" t="str">
         <v>Start Date</v>
       </c>
-      <c r="S1" s="3" t="str">
+      <c r="W1" s="3" t="str">
         <v>Discontinued Date</v>
       </c>
-      <c r="T1" s="3" t="str">
+      <c r="X1" s="3" t="str">
+        <v>Vendor Attributes (JSON)</v>
+      </c>
+      <c r="Y1" s="3" t="str">
         <v>Diff Status</v>
       </c>
-      <c r="U1" s="3" t="str">
+      <c r="Z1" s="3" t="str">
         <v>Previous List Price (USD)</v>
       </c>
-      <c r="V1" s="3" t="str">
+      <c r="AA1" s="3" t="str">
         <v>Price Change (USD)</v>
       </c>
-      <c r="W1" s="3" t="str">
+      <c r="AB1" s="3" t="str">
         <v>Price Change (%)</v>
       </c>
-      <c r="X1" s="3" t="str">
+      <c r="AC1" s="3" t="str">
         <v>Price History Trail</v>
       </c>
     </row>
@@ -1398,24 +1483,39 @@
         <v>Yes</v>
       </c>
       <c r="R2" s="2" t="str">
+        <v/>
+      </c>
+      <c r="S2" s="2" t="str">
+        <v/>
+      </c>
+      <c r="T2" s="2" t="str">
+        <v/>
+      </c>
+      <c r="U2" s="2" t="str">
+        <v/>
+      </c>
+      <c r="V2" s="2" t="str">
         <v>—</v>
       </c>
-      <c r="S2" s="2" t="str">
-        <v/>
-      </c>
-      <c r="T2" s="2" t="str">
+      <c r="W2" s="2" t="str">
+        <v/>
+      </c>
+      <c r="X2" s="2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" s="2" t="str">
         <v>UNCHANGED</v>
       </c>
-      <c r="U2" s="6">
+      <c r="Z2" s="6">
         <v>12500</v>
       </c>
-      <c r="V2" s="6">
-        <v>0</v>
-      </c>
-      <c r="W2" s="6">
-        <v>0</v>
-      </c>
-      <c r="X2" s="6">
+      <c r="AA2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB2" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC2" s="6">
         <v>2026</v>
       </c>
     </row>
@@ -1472,24 +1572,39 @@
         <v>Yes</v>
       </c>
       <c r="R3" s="2" t="str">
+        <v/>
+      </c>
+      <c r="S3" s="2" t="str">
+        <v/>
+      </c>
+      <c r="T3" s="2" t="str">
+        <v/>
+      </c>
+      <c r="U3" s="2" t="str">
+        <v/>
+      </c>
+      <c r="V3" s="2" t="str">
         <v>—</v>
       </c>
-      <c r="S3" s="2" t="str">
-        <v/>
-      </c>
-      <c r="T3" s="2" t="str">
+      <c r="W3" s="2" t="str">
+        <v/>
+      </c>
+      <c r="X3" s="2" t="str">
+        <v/>
+      </c>
+      <c r="Y3" s="2" t="str">
         <v>UNCHANGED</v>
       </c>
-      <c r="U3" s="6">
+      <c r="Z3" s="6">
         <v>18900</v>
       </c>
-      <c r="V3" s="6">
-        <v>0</v>
-      </c>
-      <c r="W3" s="6">
-        <v>0</v>
-      </c>
-      <c r="X3" s="6">
+      <c r="AA3" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC3" s="6">
         <v>2026</v>
       </c>
     </row>
@@ -1546,31 +1661,46 @@
         <v>Yes</v>
       </c>
       <c r="R4" s="2" t="str">
+        <v/>
+      </c>
+      <c r="S4" s="2" t="str">
+        <v/>
+      </c>
+      <c r="T4" s="2" t="str">
+        <v/>
+      </c>
+      <c r="U4" s="2" t="str">
+        <v/>
+      </c>
+      <c r="V4" s="2" t="str">
         <v>—</v>
       </c>
-      <c r="S4" s="2" t="str">
-        <v/>
-      </c>
-      <c r="T4" s="2" t="str">
+      <c r="W4" s="2" t="str">
+        <v/>
+      </c>
+      <c r="X4" s="2" t="str">
+        <v/>
+      </c>
+      <c r="Y4" s="2" t="str">
         <v>UNCHANGED</v>
       </c>
-      <c r="U4" s="6">
+      <c r="Z4" s="6">
         <v>15200</v>
       </c>
-      <c r="V4" s="6">
-        <v>0</v>
-      </c>
-      <c r="W4" s="6">
-        <v>0</v>
-      </c>
-      <c r="X4" s="6">
+      <c r="AA4" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="6">
         <v>2026</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X4"/>
+  <autoFilter ref="A1:AC4"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:X4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix(registry): align SCRAPED_CATALOGS columns, auto-detect learned rules, and harden catalog sync
- Add INV-133 through INV-137 to docs/INVARIANTS.md
- Fix column misalignment in outputs/SCRAPED_CATALOGS.md by adding Learned Rules header and migrating all rows to 11 columns
- Auto-detect learnedCount in scripts/lib/catalog/registry.js from catalog_deltas.json
- Make parseRegistryMD in scripts/catalogs/sync_all_registered_catalogs.js resolve outputDirMatch dynamically, preventing silent skipping across 10- vs 11-column tables
- Resync all 12 registered catalogs, generating missing Master_Catalog.csv files and refreshing diffs
- 21/21 scraping domain suites PASSED (100.0%) | 0 lint warnings/errors | CC <= 135
</commit_message>
<xml_diff>
--- a/outputs/Alletra/Storage/Alletra_Storage_System/Alletra_Storage_System_OCA_Catalog.xlsx
+++ b/outputs/Alletra/Storage/Alletra_Storage_System/Alletra_Storage_System_OCA_Catalog.xlsx
@@ -6,19 +6,21 @@
     <sheet name="Category Summary" sheetId="1" r:id="rId1"/>
     <sheet name="All SKUs" sheetId="2" r:id="rId2"/>
     <sheet name="Chassis Variants" sheetId="3" r:id="rId3"/>
-    <sheet name="Rules &amp; Constraints" sheetId="4" r:id="rId4"/>
-    <sheet name="Price History Timeline" sheetId="5" r:id="rId5"/>
-    <sheet name="Chassis" sheetId="6" r:id="rId6"/>
-    <sheet name="Metadata" sheetId="7" r:id="rId7"/>
+    <sheet name="Chassis Options Matrix" sheetId="4" r:id="rId4"/>
+    <sheet name="Rules &amp; Constraints" sheetId="5" r:id="rId5"/>
+    <sheet name="Price History Timeline" sheetId="6" r:id="rId6"/>
+    <sheet name="Chassis" sheetId="7" r:id="rId7"/>
+    <sheet name="Metadata" sheetId="8" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Category Summary'!A1:H2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">'All SKUs'!A1:AC4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2">'Chassis Variants'!A1:K4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3">'Rules &amp; Constraints'!A1:E3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4">'Price History Timeline'!A1:G4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5">'Chassis'!A1:AC4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6">'Metadata'!A1:B21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2">'Chassis Variants'!A1:L4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3">'Chassis Options Matrix'!A1:M4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4">'Rules &amp; Constraints'!A1:E3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5">'Price History Timeline'!A1:G4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6">'Chassis'!A1:AC4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7">'Metadata'!A1:B22</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -50,7 +52,7 @@
   <numFmts count="1">
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -83,8 +85,20 @@
       <b/>
       <color rgb="FFFFFFFF"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -119,6 +133,18 @@
         <bgColor/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF004B87"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF004B87"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -139,7 +165,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -155,6 +181,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -733,7 +765,7 @@
         <v/>
       </c>
       <c r="Q2" s="2" t="str">
-        <v>Yes</v>
+        <v>Unknown</v>
       </c>
       <c r="R2" s="2" t="str">
         <v/>
@@ -822,7 +854,7 @@
         <v/>
       </c>
       <c r="Q3" s="2" t="str">
-        <v>Yes</v>
+        <v>Unknown</v>
       </c>
       <c r="R3" s="2" t="str">
         <v/>
@@ -911,7 +943,7 @@
         <v/>
       </c>
       <c r="Q4" s="2" t="str">
-        <v>Yes</v>
+        <v>Unknown</v>
       </c>
       <c r="R4" s="2" t="str">
         <v/>
@@ -960,19 +992,20 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:L4"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
     <col min="3" max="3" width="75.83203125" customWidth="1"/>
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="40.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="100.83203125" customWidth="1"/>
-    <col min="11" max="11" width="80.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="40.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="100.83203125" customWidth="1"/>
+    <col min="12" max="12" width="80.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -989,24 +1022,27 @@
         <v>Option Type</v>
       </c>
       <c r="E1" s="8" t="str">
+        <v>HPE Recommended</v>
+      </c>
+      <c r="F1" s="8" t="str">
         <v>List Price (USD)</v>
       </c>
-      <c r="F1" s="8" t="str">
+      <c r="G1" s="8" t="str">
         <v>Constraint</v>
       </c>
-      <c r="G1" s="8" t="str">
+      <c r="H1" s="8" t="str">
         <v>Start Date</v>
       </c>
-      <c r="H1" s="8" t="str">
+      <c r="I1" s="8" t="str">
         <v>Discontinued Date</v>
       </c>
-      <c r="I1" s="8" t="str">
+      <c r="J1" s="8" t="str">
         <v>Diff Status</v>
       </c>
-      <c r="J1" s="8" t="str">
+      <c r="K1" s="8" t="str">
         <v>Price History Trail</v>
       </c>
-      <c r="K1" s="8" t="str">
+      <c r="L1" s="8" t="str">
         <v>Note</v>
       </c>
     </row>
@@ -1023,25 +1059,28 @@
       <c r="D2" s="2" t="str">
         <v>CTO</v>
       </c>
-      <c r="E2" s="6">
+      <c r="E2" s="2" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="F2" s="6">
         <v>12500</v>
       </c>
-      <c r="F2" s="2" t="str">
+      <c r="G2" s="2" t="str">
         <v>max 1</v>
       </c>
-      <c r="G2" s="2" t="str">
+      <c r="H2" s="2" t="str">
         <v>—</v>
       </c>
-      <c r="H2" s="2" t="str">
-        <v>Active</v>
-      </c>
       <c r="I2" s="2" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="J2" s="2" t="str">
         <v>UNCHANGED</v>
       </c>
-      <c r="J2" s="6">
+      <c r="K2" s="6">
         <v>2026</v>
       </c>
-      <c r="K2" s="2" t="str">
+      <c r="L2" s="2" t="str">
         <v>Select ONE chassis variant as the mandatory CTO base. All component rules, drive bay limits, and power constraints depend on this selection.</v>
       </c>
     </row>
@@ -1058,25 +1097,28 @@
       <c r="D3" s="2" t="str">
         <v>CTO</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="2" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="F3" s="6">
         <v>18900</v>
       </c>
-      <c r="F3" s="2" t="str">
+      <c r="G3" s="2" t="str">
         <v>max 1</v>
       </c>
-      <c r="G3" s="2" t="str">
+      <c r="H3" s="2" t="str">
         <v>—</v>
       </c>
-      <c r="H3" s="2" t="str">
-        <v>Active</v>
-      </c>
       <c r="I3" s="2" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="J3" s="2" t="str">
         <v>UNCHANGED</v>
       </c>
-      <c r="J3" s="6">
+      <c r="K3" s="6">
         <v>2026</v>
       </c>
-      <c r="K3" s="2" t="str">
+      <c r="L3" s="2" t="str">
         <v>Select ONE chassis variant as the mandatory CTO base. All component rules, drive bay limits, and power constraints depend on this selection.</v>
       </c>
     </row>
@@ -1093,37 +1135,231 @@
       <c r="D4" s="2" t="str">
         <v>CTO</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="2" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="F4" s="6">
         <v>15200</v>
       </c>
-      <c r="F4" s="2" t="str">
+      <c r="G4" s="2" t="str">
         <v>max 1</v>
       </c>
-      <c r="G4" s="2" t="str">
+      <c r="H4" s="2" t="str">
         <v>—</v>
       </c>
-      <c r="H4" s="2" t="str">
-        <v>Active</v>
-      </c>
       <c r="I4" s="2" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="J4" s="2" t="str">
         <v>UNCHANGED</v>
       </c>
-      <c r="J4" s="6">
+      <c r="K4" s="6">
         <v>2026</v>
       </c>
-      <c r="K4" s="2" t="str">
+      <c r="L4" s="2" t="str">
         <v>Select ONE chassis variant as the mandatory CTO base. All component rules, drive bay limits, and power constraints depend on this selection.</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K4"/>
+  <autoFilter ref="A1:L4"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M4"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="35.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
+    <col min="8" max="8" width="55.83203125" customWidth="1"/>
+    <col min="9" max="9" width="40.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="18.83203125" customWidth="1"/>
+    <col min="13" max="13" width="80.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="str">
+        <v>Base SKU</v>
+      </c>
+      <c r="B1" s="10" t="str">
+        <v>Form Factor</v>
+      </c>
+      <c r="C1" s="10" t="str">
+        <v>Option Type</v>
+      </c>
+      <c r="D1" s="10" t="str">
+        <v>HPE Recommended</v>
+      </c>
+      <c r="E1" s="10" t="str">
+        <v>List Price (USD)</v>
+      </c>
+      <c r="F1" s="10" t="str">
+        <v>Drive Media Supported</v>
+      </c>
+      <c r="G1" s="10" t="str">
+        <v>Base Drive Bays</v>
+      </c>
+      <c r="H1" s="10" t="str">
+        <v>Max Expandability</v>
+      </c>
+      <c r="I1" s="10" t="str">
+        <v>Power Envelope</v>
+      </c>
+      <c r="J1" s="10" t="str">
+        <v>Lifecycle Status</v>
+      </c>
+      <c r="K1" s="10" t="str">
+        <v>Start Date</v>
+      </c>
+      <c r="L1" s="10" t="str">
+        <v>Discontinued Date</v>
+      </c>
+      <c r="M1" s="10" t="str">
+        <v>Architectural Rules</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="str">
+        <v>R0Q35A</v>
+      </c>
+      <c r="B2" s="2" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="C2" s="2" t="str">
+        <v>CTO</v>
+      </c>
+      <c r="D2" s="2" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="E2" s="6">
+        <v>12500</v>
+      </c>
+      <c r="F2" s="2" t="str">
+        <v>UNVERIFIED — variant-specific evidence required</v>
+      </c>
+      <c r="G2" s="2" t="str">
+        <v>UNVERIFIED — title is not a bay inventory</v>
+      </c>
+      <c r="H2" s="2" t="str">
+        <v>UNVERIFIED — variant-specific evidence required</v>
+      </c>
+      <c r="I2" s="2" t="str">
+        <v>UNVERIFIED — variant-specific evidence required</v>
+      </c>
+      <c r="J2" s="2" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="K2" s="2" t="str">
+        <v>—</v>
+      </c>
+      <c r="L2" s="2" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="M2" s="2" t="str">
+        <v>NOT VERIFIED: do not transfer compatibility or rules between base SKUs without scoped vendor evidence.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="str">
+        <v>R0Q36A</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="C3" s="2" t="str">
+        <v>CTO</v>
+      </c>
+      <c r="D3" s="2" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="E3" s="6">
+        <v>18900</v>
+      </c>
+      <c r="F3" s="2" t="str">
+        <v>UNVERIFIED — variant-specific evidence required</v>
+      </c>
+      <c r="G3" s="2" t="str">
+        <v>UNVERIFIED — title is not a bay inventory</v>
+      </c>
+      <c r="H3" s="2" t="str">
+        <v>UNVERIFIED — variant-specific evidence required</v>
+      </c>
+      <c r="I3" s="2" t="str">
+        <v>UNVERIFIED — variant-specific evidence required</v>
+      </c>
+      <c r="J3" s="2" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="K3" s="2" t="str">
+        <v>—</v>
+      </c>
+      <c r="L3" s="2" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="M3" s="2" t="str">
+        <v>NOT VERIFIED: do not transfer compatibility or rules between base SKUs without scoped vendor evidence.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="str">
+        <v>R0Q37A</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="C4" s="2" t="str">
+        <v>CTO</v>
+      </c>
+      <c r="D4" s="2" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="E4" s="6">
+        <v>15200</v>
+      </c>
+      <c r="F4" s="2" t="str">
+        <v>UNVERIFIED — variant-specific evidence required</v>
+      </c>
+      <c r="G4" s="2" t="str">
+        <v>UNVERIFIED — title is not a bay inventory</v>
+      </c>
+      <c r="H4" s="2" t="str">
+        <v>UNVERIFIED — variant-specific evidence required</v>
+      </c>
+      <c r="I4" s="2" t="str">
+        <v>UNVERIFIED — variant-specific evidence required</v>
+      </c>
+      <c r="J4" s="2" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="K4" s="2" t="str">
+        <v>—</v>
+      </c>
+      <c r="L4" s="2" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="M4" s="2" t="str">
+        <v>NOT VERIFIED: do not transfer compatibility or rules between base SKUs without scoped vendor evidence.</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M4"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E3"/>
   <cols>
@@ -1193,7 +1429,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G4"/>
   <cols>
@@ -1306,7 +1542,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AC4"/>
   <cols>
@@ -1480,7 +1716,7 @@
         <v/>
       </c>
       <c r="Q2" s="2" t="str">
-        <v>Yes</v>
+        <v>Unknown</v>
       </c>
       <c r="R2" s="2" t="str">
         <v/>
@@ -1569,7 +1805,7 @@
         <v/>
       </c>
       <c r="Q3" s="2" t="str">
-        <v>Yes</v>
+        <v>Unknown</v>
       </c>
       <c r="R3" s="2" t="str">
         <v/>
@@ -1658,7 +1894,7 @@
         <v/>
       </c>
       <c r="Q4" s="2" t="str">
-        <v>Yes</v>
+        <v>Unknown</v>
       </c>
       <c r="R4" s="2" t="str">
         <v/>
@@ -1705,9 +1941,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="80.83203125" customWidth="1"/>
@@ -1795,23 +2031,23 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="str">
-        <v>Total Tables</v>
+        <v>Unavailable DOM Rules</v>
       </c>
       <c r="B11" s="2" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="str">
-        <v>Diff Added SKUs</v>
+        <v>Total Tables</v>
       </c>
       <c r="B12" s="2" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="str">
-        <v>Diff Removed SKUs</v>
+        <v>Diff Added SKUs</v>
       </c>
       <c r="B13" s="2" t="str">
         <v>0</v>
@@ -1819,7 +2055,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="str">
-        <v>Diff Price Changed</v>
+        <v>Diff Removed SKUs</v>
       </c>
       <c r="B14" s="2" t="str">
         <v>0</v>
@@ -1827,7 +2063,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="str">
-        <v>Diff Attr Changed</v>
+        <v>Diff Price Changed</v>
       </c>
       <c r="B15" s="2" t="str">
         <v>0</v>
@@ -1835,7 +2071,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="str">
-        <v>Diff Reinstated SKUs</v>
+        <v>Diff Attr Changed</v>
       </c>
       <c r="B16" s="2" t="str">
         <v>0</v>
@@ -1843,23 +2079,23 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="str">
-        <v>Diff Unchanged SKUs</v>
+        <v>Diff Reinstated SKUs</v>
       </c>
       <c r="B17" s="2" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="str">
-        <v>Discontinued (All-Time)</v>
+        <v>Diff Unchanged SKUs</v>
       </c>
       <c r="B18" s="2" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="str">
-        <v>Reinstated (All-Time)</v>
+        <v>Discontinued (All-Time)</v>
       </c>
       <c r="B19" s="2" t="str">
         <v>0</v>
@@ -1867,24 +2103,32 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="str">
-        <v>Services JSON</v>
+        <v>Reinstated (All-Time)</v>
       </c>
       <c r="B20" s="2" t="str">
-        <v>(Not yet generated)</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="str">
+        <v>Services JSON</v>
+      </c>
+      <c r="B21" s="2" t="str">
+        <v>(Not yet generated)</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="str">
         <v>Output Folder</v>
       </c>
-      <c r="B21" s="2" t="str">
-        <v>/home/vinodh/vendorNotebookSolution/outputs/Alletra/Storage/Alletra_Storage_System</v>
+      <c r="B22" s="2" t="str">
+        <v>C:\Users\latha\.gemini\antigravity\scratch\antigravityProjects\updatedVendorScrapingNotebook-v2\outputs\Alletra\Storage\Alletra_Storage_System</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B21"/>
+  <autoFilter ref="A1:B22"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>